<commit_message>
Bring in stress-in-action content (20260327 release)
Tree set to stress-in-action/sia.project.1.wd.data@c561d0e: updated raw
tables, 05.ui_constants.R, library(shiny), full 20260327 processed set.
Drops the 20260227 processed files (kept in history).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/data_access.xlsx
+++ b/data/raw/data_access.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\msa583\Downloads\Relational Database_26-02-2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zxu567\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4484C9E1-62F9-40C9-8CD2-6210A6186303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C05EC263-E747-450C-9A42-54BC239EC507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7A7D6C86-A6AC-403C-91E2-C0E7310CD44B}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2530" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2929" uniqueCount="345">
   <si>
     <t>device_id</t>
   </si>
@@ -931,6 +931,151 @@
   </si>
   <si>
     <t>Omnisense software</t>
+  </si>
+  <si>
+    <t>046_sia_wd_rin</t>
+  </si>
+  <si>
+    <t>Activity intensity, HR, HRV, RR, SpO2, Skin Temperature, Slepp Stages, Sleep Apnea Detection, Steps, Stress Index</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1min: SpO2, 5min: HR, 1 hour: activity intensity, sleep stages, steps  </t>
+  </si>
+  <si>
+    <t>Bluetooth 5.0; Low power bluetooth module</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes </t>
+  </si>
+  <si>
+    <t>RingConn App</t>
+  </si>
+  <si>
+    <t>Apple Health, Google Fit or others to keep your data for longer</t>
+  </si>
+  <si>
+    <t>United Kingdom for users in the United States, the United Kingdom and the European Economic Area (EEA), and servers in People's Republic of China for users in People's Republic of China.</t>
+  </si>
+  <si>
+    <t>047_sia_wd_ult</t>
+  </si>
+  <si>
+    <t>HR;Sleep stages (with REM); Sleep efficiency score; Sleep restfulness score; Sleep time; HRV-RMSSD; HRV-SDNN; Stress score; Step Count; Distance; EE; VO2max; Atrial Fibrillation detection; Cardio Adaptability detection; Circadian Alignment Suggestions; RR; Blood oxygen saturation; Dynamic recovery score; Sleep movements; Movement score; Active minutes; Workout frequency; Detection of Stress periods; Detection of Relaxed periods; Detection of Stimulated periods; Detection of Active periods; Resting heart rate; Skin temp</t>
+  </si>
+  <si>
+    <t>5min: HRV; 30min: HR, Active minutes, Stress score; 1hour: Sleep movements; 1day: Sleep stages (with REM); Sleep efficiency score; Sleep restfulness score; Sleep time</t>
+  </si>
+  <si>
+    <t>Bluethooth low energy (BLE5)</t>
+  </si>
+  <si>
+    <t>Android 6 or later</t>
+  </si>
+  <si>
+    <t>iOS 15 or later</t>
+  </si>
+  <si>
+    <t>Ultrahuman App</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U.S., possibly india </t>
+  </si>
+  <si>
+    <t xml:space="preserve">it is mentioned that data can be collected, stored, and used in any country the company operates in, which is in India and therefore, not GDPR compliant </t>
+  </si>
+  <si>
+    <t>048_sia_wd_nua</t>
+  </si>
+  <si>
+    <t>DNE (Propriatory Nuanic index (1-100) derived from EDA and accelerometry)</t>
+  </si>
+  <si>
+    <t>1min: DNE</t>
+  </si>
+  <si>
+    <t>Bluetooth LE</t>
+  </si>
+  <si>
+    <t>Android 5 or higher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">iOS 14 or higher </t>
+  </si>
+  <si>
+    <t>Nuanic App</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nuanic Could will become available and will be GDPR compliant with data stored within the European Economic Area. Data might me processed outside of this area. Could storage will be optional and the integrated storage can still be used.  </t>
+  </si>
+  <si>
+    <t>data can be stored directly on the mobile device that runs the app</t>
+  </si>
+  <si>
+    <t>049_sia_wd_cos</t>
+  </si>
+  <si>
+    <t>Core Temperature; HR; RR; SpO2</t>
+  </si>
+  <si>
+    <t>c-med° App, and Cosinuss Health App0</t>
+  </si>
+  <si>
+    <t>Cosinuss Lab system</t>
+  </si>
+  <si>
+    <t>050_sia_wd_lum</t>
+  </si>
+  <si>
+    <t>Blood flow to the head; HR; HRV; Daily average flow index; Daily minimum flow index</t>
+  </si>
+  <si>
+    <t>5min: all</t>
+  </si>
+  <si>
+    <t>iOS 16 or later</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lumia: Manage your dizziness app (available in US only) </t>
+  </si>
+  <si>
+    <t>051_sia_wd_plu</t>
+  </si>
+  <si>
+    <t>Breathing cycle amplitude parameters (max, mean, SD, root-mean-square and total energy estimation); breathing frequency parameters; RR; Breath-to-Breath Interval (BBI) parameters (min, max, mean, SD  root-mean-square and total BBI differences); 
+HRV parameters (SDNN, RMSSD, NN20, pNN20, pNN50); mean HR; NN50; ECG frequency parameters (VLF, LF, HF, peak frequency, absolute powers, normalized powers, LF/HF ratio);
+EMG activation-specific parameters (start, end, duration of muscle activation, latency, peak-to-peak amplitudes, root-mean-square, integral over activation segment);
+electrodermal response (EDR) latency; EDR amplitude, EDR rise time; EDR recovery time (to 50% and to 63% of EDR amplitude); Response peak after stimulus, total power estimation;
+maximum foce (N); force reproduction rate; jump height; fleight time during jump</t>
+  </si>
+  <si>
+    <t>Bluetooth 2.0+EDR, USB calbe to download stored data from memory (optional extra)</t>
+  </si>
+  <si>
+    <t>OepnSignals (r)evolution</t>
+  </si>
+  <si>
+    <t xml:space="preserve">default is 0 internal storage, but optionally available </t>
+  </si>
+  <si>
+    <t>052_sia_wd_plu</t>
+  </si>
+  <si>
+    <t>RR; breath-to-breath interval parameters (Minimum, maximum, mean, standard deviation &amp; root-mean-square of successive BBI differences); Breathing cycle amplitude parameters (Maximum, mean, standard deviation, root-mean-square &amp; total energy estimation); frequency parameters</t>
+  </si>
+  <si>
+    <t>Bluetooth required to transfer from device to phone; Flexible methods to transfer from phone application to computer.</t>
+  </si>
+  <si>
+    <t>for OpenSignals anlyses software</t>
+  </si>
+  <si>
+    <t>for Biosignals Studio Mobile Recording software</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biosignals Studio </t>
+  </si>
+  <si>
+    <t>OpenSignals</t>
   </si>
 </sst>
 </file>
@@ -1075,7 +1220,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1130,6 +1275,9 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1465,7 +1613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA1BD5DC-A81B-4D9C-8626-3C643AFB0E7B}">
-  <dimension ref="A1:F766"/>
+  <dimension ref="A1:F886"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="16.5546875" customWidth="1"/>
@@ -10938,6 +11086,1485 @@
       <c r="D766" s="10"/>
       <c r="E766" s="10"/>
       <c r="F766" s="21"/>
+    </row>
+    <row r="767" spans="1:6">
+      <c r="A767" t="s">
+        <v>0</v>
+      </c>
+      <c r="B767" t="s">
+        <v>1</v>
+      </c>
+      <c r="C767" t="s">
+        <v>2</v>
+      </c>
+      <c r="D767" t="s">
+        <v>3</v>
+      </c>
+      <c r="E767" t="s">
+        <v>4</v>
+      </c>
+      <c r="F767" s="14" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="768" spans="1:6">
+      <c r="A768" t="s">
+        <v>298</v>
+      </c>
+      <c r="B768" t="s">
+        <v>7</v>
+      </c>
+      <c r="C768" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="769" spans="1:6">
+      <c r="A769" t="s">
+        <v>298</v>
+      </c>
+      <c r="B769" t="s">
+        <v>9</v>
+      </c>
+      <c r="F769" s="14" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="770" spans="1:6">
+      <c r="A770" t="s">
+        <v>298</v>
+      </c>
+      <c r="B770" t="s">
+        <v>11</v>
+      </c>
+      <c r="F770" s="14" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="771" spans="1:6">
+      <c r="A771" t="s">
+        <v>298</v>
+      </c>
+      <c r="B771" t="s">
+        <v>12</v>
+      </c>
+      <c r="C771" t="s">
+        <v>8</v>
+      </c>
+      <c r="F771" s="14" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="772" spans="1:6">
+      <c r="A772" t="s">
+        <v>298</v>
+      </c>
+      <c r="B772" t="s">
+        <v>14</v>
+      </c>
+      <c r="C772" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="773" spans="1:6">
+      <c r="A773" t="s">
+        <v>298</v>
+      </c>
+      <c r="B773" t="s">
+        <v>16</v>
+      </c>
+      <c r="C773" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="774" spans="1:6">
+      <c r="A774" t="s">
+        <v>298</v>
+      </c>
+      <c r="B774" t="s">
+        <v>17</v>
+      </c>
+      <c r="C774" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="775" spans="1:6">
+      <c r="A775" t="s">
+        <v>298</v>
+      </c>
+      <c r="B775" t="s">
+        <v>19</v>
+      </c>
+      <c r="C775" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="776" spans="1:6">
+      <c r="A776" t="s">
+        <v>298</v>
+      </c>
+      <c r="B776" t="s">
+        <v>21</v>
+      </c>
+      <c r="C776" t="s">
+        <v>302</v>
+      </c>
+      <c r="F776" s="14" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="777" spans="1:6">
+      <c r="A777" t="s">
+        <v>298</v>
+      </c>
+      <c r="B777" t="s">
+        <v>23</v>
+      </c>
+      <c r="C777" t="s">
+        <v>8</v>
+      </c>
+      <c r="F777" s="14" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="778" spans="1:6">
+      <c r="A778" t="s">
+        <v>298</v>
+      </c>
+      <c r="B778" t="s">
+        <v>25</v>
+      </c>
+      <c r="C778" t="s">
+        <v>302</v>
+      </c>
+      <c r="F778" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="779" spans="1:6">
+      <c r="A779" t="s">
+        <v>298</v>
+      </c>
+      <c r="B779" t="s">
+        <v>27</v>
+      </c>
+      <c r="C779" t="s">
+        <v>8</v>
+      </c>
+      <c r="F779" s="14" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="780" spans="1:6">
+      <c r="A780" t="s">
+        <v>298</v>
+      </c>
+      <c r="B780" t="s">
+        <v>29</v>
+      </c>
+      <c r="D780">
+        <v>168</v>
+      </c>
+      <c r="E780" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="781" spans="1:6">
+      <c r="A781" t="s">
+        <v>298</v>
+      </c>
+      <c r="B781" t="s">
+        <v>31</v>
+      </c>
+      <c r="D781">
+        <v>-9999</v>
+      </c>
+      <c r="E781" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="782" spans="1:6">
+      <c r="A782" t="s">
+        <v>298</v>
+      </c>
+      <c r="B782" t="s">
+        <v>33</v>
+      </c>
+      <c r="C782" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="783" spans="1:6">
+      <c r="A783" t="s">
+        <v>298</v>
+      </c>
+      <c r="B783" t="s">
+        <v>34</v>
+      </c>
+      <c r="C783" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="784" spans="1:6">
+      <c r="A784" t="s">
+        <v>298</v>
+      </c>
+      <c r="B784" t="s">
+        <v>36</v>
+      </c>
+      <c r="C784" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="785" spans="1:6">
+      <c r="A785" t="s">
+        <v>306</v>
+      </c>
+      <c r="B785" t="s">
+        <v>7</v>
+      </c>
+      <c r="C785" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="786" spans="1:6">
+      <c r="A786" t="s">
+        <v>306</v>
+      </c>
+      <c r="B786" t="s">
+        <v>9</v>
+      </c>
+      <c r="F786" s="14" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="787" spans="1:6">
+      <c r="A787" t="s">
+        <v>306</v>
+      </c>
+      <c r="B787" t="s">
+        <v>11</v>
+      </c>
+      <c r="F787" s="14" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="788" spans="1:6">
+      <c r="A788" t="s">
+        <v>306</v>
+      </c>
+      <c r="B788" t="s">
+        <v>12</v>
+      </c>
+      <c r="C788" t="s">
+        <v>8</v>
+      </c>
+      <c r="F788" s="14" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="789" spans="1:6">
+      <c r="A789" t="s">
+        <v>306</v>
+      </c>
+      <c r="B789" t="s">
+        <v>14</v>
+      </c>
+      <c r="C789" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="790" spans="1:6">
+      <c r="A790" t="s">
+        <v>306</v>
+      </c>
+      <c r="B790" t="s">
+        <v>16</v>
+      </c>
+      <c r="C790" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="791" spans="1:6">
+      <c r="A791" t="s">
+        <v>306</v>
+      </c>
+      <c r="B791" t="s">
+        <v>17</v>
+      </c>
+      <c r="C791" t="s">
+        <v>8</v>
+      </c>
+      <c r="F791" s="14" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="792" spans="1:6">
+      <c r="A792" t="s">
+        <v>306</v>
+      </c>
+      <c r="B792" t="s">
+        <v>19</v>
+      </c>
+      <c r="C792" t="s">
+        <v>8</v>
+      </c>
+      <c r="F792" s="14" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="793" spans="1:6">
+      <c r="A793" t="s">
+        <v>306</v>
+      </c>
+      <c r="B793" t="s">
+        <v>21</v>
+      </c>
+      <c r="C793" t="s">
+        <v>8</v>
+      </c>
+      <c r="F793" s="14" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="794" spans="1:6">
+      <c r="A794" t="s">
+        <v>306</v>
+      </c>
+      <c r="B794" t="s">
+        <v>23</v>
+      </c>
+      <c r="C794" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="795" spans="1:6">
+      <c r="A795" t="s">
+        <v>306</v>
+      </c>
+      <c r="B795" t="s">
+        <v>25</v>
+      </c>
+      <c r="C795" t="s">
+        <v>8</v>
+      </c>
+      <c r="F795" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="796" spans="1:6">
+      <c r="A796" t="s">
+        <v>306</v>
+      </c>
+      <c r="B796" t="s">
+        <v>27</v>
+      </c>
+      <c r="C796" t="s">
+        <v>8</v>
+      </c>
+      <c r="F796" s="14" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="797" spans="1:6">
+      <c r="A797" t="s">
+        <v>306</v>
+      </c>
+      <c r="B797" t="s">
+        <v>29</v>
+      </c>
+      <c r="D797">
+        <v>168</v>
+      </c>
+      <c r="E797" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="798" spans="1:6">
+      <c r="A798" t="s">
+        <v>306</v>
+      </c>
+      <c r="B798" t="s">
+        <v>31</v>
+      </c>
+      <c r="D798">
+        <v>-9999</v>
+      </c>
+      <c r="E798" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="799" spans="1:6">
+      <c r="A799" t="s">
+        <v>306</v>
+      </c>
+      <c r="B799" t="s">
+        <v>33</v>
+      </c>
+      <c r="C799" t="s">
+        <v>35</v>
+      </c>
+      <c r="F799" s="14" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="800" spans="1:6">
+      <c r="A800" t="s">
+        <v>306</v>
+      </c>
+      <c r="B800" t="s">
+        <v>34</v>
+      </c>
+      <c r="C800" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="801" spans="1:6">
+      <c r="A801" t="s">
+        <v>306</v>
+      </c>
+      <c r="B801" t="s">
+        <v>36</v>
+      </c>
+      <c r="C801" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="802" spans="1:6">
+      <c r="A802" t="s">
+        <v>315</v>
+      </c>
+      <c r="B802" t="s">
+        <v>7</v>
+      </c>
+      <c r="C802" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="803" spans="1:6">
+      <c r="A803" t="s">
+        <v>315</v>
+      </c>
+      <c r="B803" t="s">
+        <v>9</v>
+      </c>
+      <c r="F803" s="14" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="804" spans="1:6">
+      <c r="A804" t="s">
+        <v>315</v>
+      </c>
+      <c r="B804" t="s">
+        <v>11</v>
+      </c>
+      <c r="F804" s="14" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="805" spans="1:6">
+      <c r="A805" t="s">
+        <v>315</v>
+      </c>
+      <c r="B805" t="s">
+        <v>12</v>
+      </c>
+      <c r="C805" t="s">
+        <v>8</v>
+      </c>
+      <c r="F805" s="14" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="806" spans="1:6">
+      <c r="A806" t="s">
+        <v>315</v>
+      </c>
+      <c r="B806" t="s">
+        <v>14</v>
+      </c>
+      <c r="C806" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="807" spans="1:6">
+      <c r="A807" t="s">
+        <v>315</v>
+      </c>
+      <c r="B807" t="s">
+        <v>16</v>
+      </c>
+      <c r="C807" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="808" spans="1:6">
+      <c r="A808" t="s">
+        <v>315</v>
+      </c>
+      <c r="B808" t="s">
+        <v>17</v>
+      </c>
+      <c r="C808" t="s">
+        <v>8</v>
+      </c>
+      <c r="F808" s="14" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="809" spans="1:6">
+      <c r="A809" t="s">
+        <v>315</v>
+      </c>
+      <c r="B809" t="s">
+        <v>19</v>
+      </c>
+      <c r="C809" t="s">
+        <v>8</v>
+      </c>
+      <c r="F809" s="14" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="810" spans="1:6">
+      <c r="A810" t="s">
+        <v>315</v>
+      </c>
+      <c r="B810" t="s">
+        <v>21</v>
+      </c>
+      <c r="C810" t="s">
+        <v>8</v>
+      </c>
+      <c r="F810" s="14" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="811" spans="1:6">
+      <c r="A811" t="s">
+        <v>315</v>
+      </c>
+      <c r="B811" t="s">
+        <v>23</v>
+      </c>
+      <c r="C811" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="812" spans="1:6">
+      <c r="A812" t="s">
+        <v>315</v>
+      </c>
+      <c r="B812" t="s">
+        <v>25</v>
+      </c>
+      <c r="C812" t="s">
+        <v>8</v>
+      </c>
+      <c r="F812" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="813" spans="1:6">
+      <c r="A813" t="s">
+        <v>315</v>
+      </c>
+      <c r="B813" t="s">
+        <v>27</v>
+      </c>
+      <c r="C813" t="s">
+        <v>35</v>
+      </c>
+      <c r="F813" s="14" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="814" spans="1:6">
+      <c r="A814" t="s">
+        <v>315</v>
+      </c>
+      <c r="B814" t="s">
+        <v>29</v>
+      </c>
+      <c r="D814">
+        <v>72</v>
+      </c>
+      <c r="E814" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="815" spans="1:6">
+      <c r="A815" t="s">
+        <v>315</v>
+      </c>
+      <c r="B815" t="s">
+        <v>31</v>
+      </c>
+      <c r="D815">
+        <v>-9999</v>
+      </c>
+      <c r="E815" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="816" spans="1:6">
+      <c r="A816" t="s">
+        <v>315</v>
+      </c>
+      <c r="B816" t="s">
+        <v>33</v>
+      </c>
+      <c r="C816" t="s">
+        <v>8</v>
+      </c>
+      <c r="F816" s="14" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="817" spans="1:6">
+      <c r="A817" t="s">
+        <v>315</v>
+      </c>
+      <c r="B817" t="s">
+        <v>34</v>
+      </c>
+      <c r="C817" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="818" spans="1:6">
+      <c r="A818" t="s">
+        <v>315</v>
+      </c>
+      <c r="B818" t="s">
+        <v>36</v>
+      </c>
+      <c r="C818" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="819" spans="1:6">
+      <c r="A819" t="s">
+        <v>324</v>
+      </c>
+      <c r="B819" t="s">
+        <v>7</v>
+      </c>
+      <c r="C819" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="820" spans="1:6">
+      <c r="A820" t="s">
+        <v>324</v>
+      </c>
+      <c r="B820" t="s">
+        <v>9</v>
+      </c>
+      <c r="F820" s="14" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="821" spans="1:6">
+      <c r="A821" t="s">
+        <v>324</v>
+      </c>
+      <c r="B821" t="s">
+        <v>11</v>
+      </c>
+      <c r="F821" s="14" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="822" spans="1:6">
+      <c r="A822" t="s">
+        <v>324</v>
+      </c>
+      <c r="B822" t="s">
+        <v>12</v>
+      </c>
+      <c r="C822" t="s">
+        <v>8</v>
+      </c>
+      <c r="F822" s="14" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="823" spans="1:6">
+      <c r="A823" t="s">
+        <v>324</v>
+      </c>
+      <c r="B823" t="s">
+        <v>14</v>
+      </c>
+      <c r="C823" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="824" spans="1:6">
+      <c r="A824" t="s">
+        <v>324</v>
+      </c>
+      <c r="B824" t="s">
+        <v>16</v>
+      </c>
+      <c r="C824" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="825" spans="1:6">
+      <c r="A825" t="s">
+        <v>324</v>
+      </c>
+      <c r="B825" t="s">
+        <v>17</v>
+      </c>
+      <c r="C825" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="826" spans="1:6">
+      <c r="A826" t="s">
+        <v>324</v>
+      </c>
+      <c r="B826" t="s">
+        <v>19</v>
+      </c>
+      <c r="C826" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="827" spans="1:6">
+      <c r="A827" t="s">
+        <v>324</v>
+      </c>
+      <c r="B827" t="s">
+        <v>21</v>
+      </c>
+      <c r="C827" t="s">
+        <v>8</v>
+      </c>
+      <c r="F827" s="14" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="828" spans="1:6">
+      <c r="A828" t="s">
+        <v>324</v>
+      </c>
+      <c r="B828" t="s">
+        <v>23</v>
+      </c>
+      <c r="C828" t="s">
+        <v>8</v>
+      </c>
+      <c r="F828" s="14" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="829" spans="1:6">
+      <c r="A829" t="s">
+        <v>324</v>
+      </c>
+      <c r="B829" t="s">
+        <v>25</v>
+      </c>
+      <c r="C829" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="830" spans="1:6">
+      <c r="A830" t="s">
+        <v>324</v>
+      </c>
+      <c r="B830" t="s">
+        <v>27</v>
+      </c>
+      <c r="C830" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="831" spans="1:6">
+      <c r="A831" t="s">
+        <v>324</v>
+      </c>
+      <c r="B831" t="s">
+        <v>29</v>
+      </c>
+      <c r="D831">
+        <v>-9999</v>
+      </c>
+      <c r="E831" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="832" spans="1:6">
+      <c r="A832" t="s">
+        <v>324</v>
+      </c>
+      <c r="B832" t="s">
+        <v>31</v>
+      </c>
+      <c r="D832">
+        <v>-9999</v>
+      </c>
+      <c r="E832" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="833" spans="1:6">
+      <c r="A833" t="s">
+        <v>324</v>
+      </c>
+      <c r="B833" t="s">
+        <v>33</v>
+      </c>
+      <c r="C833" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="834" spans="1:6">
+      <c r="A834" t="s">
+        <v>324</v>
+      </c>
+      <c r="B834" t="s">
+        <v>34</v>
+      </c>
+      <c r="C834" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="835" spans="1:6">
+      <c r="A835" t="s">
+        <v>324</v>
+      </c>
+      <c r="B835" t="s">
+        <v>36</v>
+      </c>
+      <c r="C835" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="836" spans="1:6">
+      <c r="A836" t="s">
+        <v>328</v>
+      </c>
+      <c r="B836" t="s">
+        <v>7</v>
+      </c>
+      <c r="C836" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="837" spans="1:6">
+      <c r="A837" t="s">
+        <v>328</v>
+      </c>
+      <c r="B837" t="s">
+        <v>9</v>
+      </c>
+      <c r="F837" s="14" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="838" spans="1:6">
+      <c r="A838" t="s">
+        <v>328</v>
+      </c>
+      <c r="B838" t="s">
+        <v>11</v>
+      </c>
+      <c r="F838" s="14" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="839" spans="1:6">
+      <c r="A839" t="s">
+        <v>328</v>
+      </c>
+      <c r="B839" t="s">
+        <v>12</v>
+      </c>
+      <c r="F839" s="14" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="840" spans="1:6">
+      <c r="A840" t="s">
+        <v>328</v>
+      </c>
+      <c r="B840" t="s">
+        <v>14</v>
+      </c>
+      <c r="C840" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="841" spans="1:6">
+      <c r="A841" t="s">
+        <v>328</v>
+      </c>
+      <c r="B841" t="s">
+        <v>16</v>
+      </c>
+      <c r="C841" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="842" spans="1:6">
+      <c r="A842" t="s">
+        <v>328</v>
+      </c>
+      <c r="B842" t="s">
+        <v>17</v>
+      </c>
+      <c r="C842" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="843" spans="1:6">
+      <c r="A843" t="s">
+        <v>328</v>
+      </c>
+      <c r="B843" t="s">
+        <v>19</v>
+      </c>
+      <c r="C843" t="s">
+        <v>8</v>
+      </c>
+      <c r="F843" s="14" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="844" spans="1:6">
+      <c r="A844" t="s">
+        <v>328</v>
+      </c>
+      <c r="B844" t="s">
+        <v>21</v>
+      </c>
+      <c r="C844" t="s">
+        <v>8</v>
+      </c>
+      <c r="F844" s="14" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="845" spans="1:6">
+      <c r="A845" t="s">
+        <v>328</v>
+      </c>
+      <c r="B845" t="s">
+        <v>23</v>
+      </c>
+      <c r="C845" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="846" spans="1:6">
+      <c r="A846" t="s">
+        <v>328</v>
+      </c>
+      <c r="B846" t="s">
+        <v>25</v>
+      </c>
+      <c r="C846" t="s">
+        <v>8</v>
+      </c>
+      <c r="F846" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="847" spans="1:6">
+      <c r="A847" t="s">
+        <v>328</v>
+      </c>
+      <c r="B847" t="s">
+        <v>27</v>
+      </c>
+      <c r="C847" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="848" spans="1:6">
+      <c r="A848" t="s">
+        <v>328</v>
+      </c>
+      <c r="B848" t="s">
+        <v>29</v>
+      </c>
+      <c r="D848">
+        <v>-9999</v>
+      </c>
+      <c r="E848" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="849" spans="1:6">
+      <c r="A849" t="s">
+        <v>328</v>
+      </c>
+      <c r="B849" t="s">
+        <v>31</v>
+      </c>
+      <c r="D849">
+        <v>-9999</v>
+      </c>
+      <c r="E849" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="850" spans="1:6">
+      <c r="A850" t="s">
+        <v>328</v>
+      </c>
+      <c r="B850" t="s">
+        <v>33</v>
+      </c>
+      <c r="C850" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="851" spans="1:6">
+      <c r="A851" t="s">
+        <v>328</v>
+      </c>
+      <c r="B851" t="s">
+        <v>34</v>
+      </c>
+      <c r="C851" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="852" spans="1:6">
+      <c r="A852" t="s">
+        <v>328</v>
+      </c>
+      <c r="B852" t="s">
+        <v>36</v>
+      </c>
+      <c r="C852" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="853" spans="1:6">
+      <c r="A853" t="s">
+        <v>333</v>
+      </c>
+      <c r="B853" t="s">
+        <v>7</v>
+      </c>
+      <c r="C853" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="854" spans="1:6">
+      <c r="A854" t="s">
+        <v>333</v>
+      </c>
+      <c r="B854" t="s">
+        <v>9</v>
+      </c>
+      <c r="F854" s="30" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="855" spans="1:6">
+      <c r="A855" t="s">
+        <v>333</v>
+      </c>
+      <c r="B855" t="s">
+        <v>11</v>
+      </c>
+      <c r="F855" s="14" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="856" spans="1:6">
+      <c r="A856" t="s">
+        <v>333</v>
+      </c>
+      <c r="B856" t="s">
+        <v>12</v>
+      </c>
+      <c r="C856" t="s">
+        <v>8</v>
+      </c>
+      <c r="F856" s="14" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="857" spans="1:6">
+      <c r="A857" t="s">
+        <v>333</v>
+      </c>
+      <c r="B857" t="s">
+        <v>14</v>
+      </c>
+      <c r="C857" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="858" spans="1:6">
+      <c r="A858" t="s">
+        <v>333</v>
+      </c>
+      <c r="B858" t="s">
+        <v>16</v>
+      </c>
+      <c r="C858" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="859" spans="1:6">
+      <c r="A859" t="s">
+        <v>333</v>
+      </c>
+      <c r="B859" t="s">
+        <v>17</v>
+      </c>
+      <c r="C859" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="860" spans="1:6">
+      <c r="A860" t="s">
+        <v>333</v>
+      </c>
+      <c r="B860" t="s">
+        <v>19</v>
+      </c>
+      <c r="C860" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="861" spans="1:6">
+      <c r="A861" t="s">
+        <v>333</v>
+      </c>
+      <c r="B861" t="s">
+        <v>21</v>
+      </c>
+      <c r="C861" t="s">
+        <v>8</v>
+      </c>
+      <c r="F861" s="14" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="862" spans="1:6">
+      <c r="A862" t="s">
+        <v>333</v>
+      </c>
+      <c r="B862" t="s">
+        <v>23</v>
+      </c>
+      <c r="C862" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="863" spans="1:6">
+      <c r="A863" t="s">
+        <v>333</v>
+      </c>
+      <c r="B863" t="s">
+        <v>25</v>
+      </c>
+      <c r="C863" t="s">
+        <v>8</v>
+      </c>
+      <c r="F863" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="864" spans="1:6">
+      <c r="A864" t="s">
+        <v>333</v>
+      </c>
+      <c r="B864" t="s">
+        <v>27</v>
+      </c>
+      <c r="C864" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="865" spans="1:6">
+      <c r="A865" t="s">
+        <v>333</v>
+      </c>
+      <c r="B865" t="s">
+        <v>29</v>
+      </c>
+      <c r="D865">
+        <v>111</v>
+      </c>
+      <c r="E865" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="866" spans="1:6">
+      <c r="A866" t="s">
+        <v>333</v>
+      </c>
+      <c r="B866" t="s">
+        <v>31</v>
+      </c>
+      <c r="D866">
+        <v>8000</v>
+      </c>
+      <c r="E866" t="s">
+        <v>32</v>
+      </c>
+      <c r="F866" s="14" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="867" spans="1:6">
+      <c r="A867" t="s">
+        <v>333</v>
+      </c>
+      <c r="B867" t="s">
+        <v>33</v>
+      </c>
+      <c r="C867" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="868" spans="1:6">
+      <c r="A868" t="s">
+        <v>333</v>
+      </c>
+      <c r="B868" t="s">
+        <v>34</v>
+      </c>
+      <c r="C868" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="869" spans="1:6">
+      <c r="A869" t="s">
+        <v>333</v>
+      </c>
+      <c r="B869" t="s">
+        <v>36</v>
+      </c>
+      <c r="C869" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="870" spans="1:6">
+      <c r="A870" t="s">
+        <v>338</v>
+      </c>
+      <c r="B870" t="s">
+        <v>7</v>
+      </c>
+      <c r="C870" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="871" spans="1:6">
+      <c r="A871" t="s">
+        <v>338</v>
+      </c>
+      <c r="B871" t="s">
+        <v>9</v>
+      </c>
+      <c r="F871" s="14" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="872" spans="1:6">
+      <c r="A872" t="s">
+        <v>338</v>
+      </c>
+      <c r="B872" t="s">
+        <v>11</v>
+      </c>
+      <c r="F872" s="14" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="873" spans="1:6">
+      <c r="A873" t="s">
+        <v>338</v>
+      </c>
+      <c r="B873" t="s">
+        <v>12</v>
+      </c>
+      <c r="C873" t="s">
+        <v>8</v>
+      </c>
+      <c r="F873" s="14" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="874" spans="1:6">
+      <c r="A874" t="s">
+        <v>338</v>
+      </c>
+      <c r="B874" t="s">
+        <v>14</v>
+      </c>
+      <c r="C874" t="s">
+        <v>8</v>
+      </c>
+      <c r="F874" s="14" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="875" spans="1:6">
+      <c r="A875" t="s">
+        <v>338</v>
+      </c>
+      <c r="B875" t="s">
+        <v>16</v>
+      </c>
+      <c r="C875" t="s">
+        <v>8</v>
+      </c>
+      <c r="F875" s="14" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="876" spans="1:6">
+      <c r="A876" t="s">
+        <v>338</v>
+      </c>
+      <c r="B876" t="s">
+        <v>17</v>
+      </c>
+      <c r="C876" t="s">
+        <v>8</v>
+      </c>
+      <c r="F876" s="14" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="877" spans="1:6">
+      <c r="A877" t="s">
+        <v>338</v>
+      </c>
+      <c r="B877" t="s">
+        <v>19</v>
+      </c>
+      <c r="C877" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="878" spans="1:6">
+      <c r="A878" t="s">
+        <v>338</v>
+      </c>
+      <c r="B878" t="s">
+        <v>21</v>
+      </c>
+      <c r="C878" t="s">
+        <v>8</v>
+      </c>
+      <c r="F878" s="14" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="879" spans="1:6">
+      <c r="A879" t="s">
+        <v>338</v>
+      </c>
+      <c r="B879" t="s">
+        <v>23</v>
+      </c>
+      <c r="C879" t="s">
+        <v>8</v>
+      </c>
+      <c r="F879" s="14" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="880" spans="1:6">
+      <c r="A880" t="s">
+        <v>338</v>
+      </c>
+      <c r="B880" t="s">
+        <v>25</v>
+      </c>
+      <c r="C880" t="s">
+        <v>8</v>
+      </c>
+      <c r="F880" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="881" spans="1:5">
+      <c r="A881" t="s">
+        <v>338</v>
+      </c>
+      <c r="B881" t="s">
+        <v>27</v>
+      </c>
+      <c r="C881" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="882" spans="1:5">
+      <c r="A882" t="s">
+        <v>338</v>
+      </c>
+      <c r="B882" t="s">
+        <v>29</v>
+      </c>
+      <c r="D882">
+        <v>10</v>
+      </c>
+      <c r="E882" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="883" spans="1:5">
+      <c r="A883" t="s">
+        <v>338</v>
+      </c>
+      <c r="B883" t="s">
+        <v>31</v>
+      </c>
+      <c r="D883">
+        <v>-9999</v>
+      </c>
+      <c r="E883" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="884" spans="1:5">
+      <c r="A884" t="s">
+        <v>338</v>
+      </c>
+      <c r="B884" t="s">
+        <v>33</v>
+      </c>
+      <c r="C884" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="885" spans="1:5">
+      <c r="A885" t="s">
+        <v>338</v>
+      </c>
+      <c r="B885" t="s">
+        <v>34</v>
+      </c>
+      <c r="C885" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="886" spans="1:5">
+      <c r="A886" t="s">
+        <v>338</v>
+      </c>
+      <c r="B886" t="s">
+        <v>36</v>
+      </c>
+      <c r="C886" t="s">
+        <v>35</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="10">
@@ -10966,17 +12593,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="71842362-ab5d-46b4-b35f-08dc9c6328ce">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8def90a7-5747-4395-b698-a599996d7912" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006131D81E7FE36E44885B3A04523FCF5D" ma:contentTypeVersion="14" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="8f9efaeda295997044994eea58453835">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="71842362-ab5d-46b4-b35f-08dc9c6328ce" xmlns:ns3="8def90a7-5747-4395-b698-a599996d7912" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7a2e7ed8b28d563a97a27396956f6ac0" ns2:_="" ns3:_="">
     <xsd:import namespace="71842362-ab5d-46b4-b35f-08dc9c6328ce"/>
@@ -11205,6 +12821,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="71842362-ab5d-46b4-b35f-08dc9c6328ce">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8def90a7-5747-4395-b698-a599996d7912" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3C3AEBB-37B4-4BFB-8F88-26E487A619B6}">
   <ds:schemaRefs>
@@ -11214,17 +12841,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EDBADEA2-FDC6-494D-BF37-E3AE079B5959}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="71842362-ab5d-46b4-b35f-08dc9c6328ce"/>
-    <ds:schemaRef ds:uri="8def90a7-5747-4395-b698-a599996d7912"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8940976A-058B-4004-A4FC-ACB49E80C650}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11241,4 +12857,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EDBADEA2-FDC6-494D-BF37-E3AE079B5959}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="71842362-ab5d-46b4-b35f-08dc9c6328ce"/>
+    <ds:schemaRef ds:uri="8def90a7-5747-4395-b698-a599996d7912"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>